<commit_message>
feat: implement product management dashboard with bulk CSV/XLSX import and CRUD functionality
</commit_message>
<xml_diff>
--- a/public/product_import_template.xlsx
+++ b/public/product_import_template.xlsx
@@ -397,17 +397,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J7"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
     <col min="3" max="3" width="15.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
     <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="10.83203125" customWidth="1"/>
     <col min="8" max="8" width="15.83203125" customWidth="1"/>
-    <col min="9" max="9" width="30.83203125" customWidth="1"/>
+    <col min="9" max="9" width="15.83203125" customWidth="1"/>
+    <col min="10" max="10" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -421,21 +422,24 @@
         <v>Category</v>
       </c>
       <c r="D1" t="str">
+        <v>Unit</v>
+      </c>
+      <c r="E1" t="str">
         <v>Unit Price</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Cost Price</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Stock</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Reorder Level</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Tax Applicable</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Description</v>
       </c>
     </row>
@@ -449,22 +453,25 @@
       <c r="C2" t="str">
         <v>Beverages</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="str">
+        <v>pcs</v>
+      </c>
+      <c r="E2">
         <v>45</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>35</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>100</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>15</v>
       </c>
-      <c r="H2" t="b">
+      <c r="I2" t="b">
         <v>1</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>Chilled soft drink bottle</v>
       </c>
     </row>
@@ -478,22 +485,25 @@
       <c r="C3" t="str">
         <v>Beverages</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="str">
+        <v>pcs</v>
+      </c>
+      <c r="E3">
         <v>40</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>32</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>80</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>10</v>
       </c>
-      <c r="H3" t="b">
+      <c r="I3" t="b">
         <v>1</v>
       </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
         <v>Chilled soft drink bottle</v>
       </c>
     </row>
@@ -507,22 +517,25 @@
       <c r="C4" t="str">
         <v>Snacks</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="str">
+        <v>pcs</v>
+      </c>
+      <c r="E4">
         <v>20</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>15</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>50</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>10</v>
       </c>
-      <c r="H4" t="b">
+      <c r="I4" t="b">
         <v>1</v>
       </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
         <v>Classic salted potato chips</v>
       </c>
     </row>
@@ -536,22 +549,25 @@
       <c r="C5" t="str">
         <v>Dairy</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="str">
+        <v>pcs</v>
+      </c>
+      <c r="E5">
         <v>60</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>52</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>30</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>5</v>
       </c>
-      <c r="H5" t="b">
+      <c r="I5" t="b">
         <v>1</v>
       </c>
-      <c r="I5" t="str">
+      <c r="J5" t="str">
         <v>Salted pasteurized butter</v>
       </c>
     </row>
@@ -565,28 +581,63 @@
       <c r="C6" t="str">
         <v>Snacks</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="str">
+        <v>pcs</v>
+      </c>
+      <c r="E6">
         <v>30</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>24</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>60</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>12</v>
       </c>
-      <c r="H6" t="b">
+      <c r="I6" t="b">
         <v>1</v>
       </c>
-      <c r="I6" t="str">
+      <c r="J6" t="str">
         <v>Chocolate cream biscuits</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Loose Basmati Rice</v>
+      </c>
+      <c r="B7" t="str">
+        <v>BASMATIRICE</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Groceries</v>
+      </c>
+      <c r="D7" t="str">
+        <v>kg</v>
+      </c>
+      <c r="E7">
+        <v>85.5</v>
+      </c>
+      <c r="F7">
+        <v>72</v>
+      </c>
+      <c r="G7">
+        <v>250.5</v>
+      </c>
+      <c r="H7">
+        <v>50</v>
+      </c>
+      <c r="I7" t="b">
+        <v>0</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Premium long grain loose basmati rice</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>